<commit_message>
seo y optimizaciones listo
</commit_message>
<xml_diff>
--- a/master.xlsx
+++ b/master.xlsx
@@ -5,21 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2f878543ae482c3e/Escritorio/Current project/03-Noarix/01-Proyectos/02-LB multiservi/web/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2f878543ae482c3e/Escritorio/Current project/03-Noarix/01-Proyectos/02-LB multiservi/web2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="495" documentId="11_AD4D2F04E46CFB4ACB3E204AFD91DD14693EDF12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4C7E2DD-55B3-4985-B63C-0AAC425AE1C5}"/>
+  <xr:revisionPtr revIDLastSave="498" documentId="11_AD4D2F04E46CFB4ACB3E204AFD91DD14693EDF12" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{742547CF-19F3-4199-870F-578760F71355}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="higuey" sheetId="1" r:id="rId1"/>
     <sheet name="extracto" sheetId="3" r:id="rId2"/>
-    <sheet name="Hoja1" sheetId="4" r:id="rId3"/>
-    <sheet name="agrupado" sheetId="2" r:id="rId4"/>
+    <sheet name="agrupado" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">agrupado!$A$7:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">agrupado!$A$7:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">extracto!$A$2:$I$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">higuey!$A$2:$G$2</definedName>
   </definedNames>
@@ -1994,7 +1993,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2037,6 +2036,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -2074,7 +2079,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -2085,16 +2090,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2110,143 +2118,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>53986</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>111705</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E55381FA-A0A6-D1D3-DAB0-37C7E2BD414C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="18281026" cy="8707065"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>21771</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>3912</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>12097</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2307DB10-3D17-22E3-5A15-AB771C213B78}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="9274628"/>
-          <a:ext cx="18281026" cy="8688012"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>98</xdr:row>
-      <xdr:rowOff>97972</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>3912</xdr:colOff>
-      <xdr:row>134</xdr:row>
-      <xdr:rowOff>75767</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A3163661-EDA0-E105-E115-3B2F54161B59}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="18233572"/>
-          <a:ext cx="18281026" cy="6639852"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14721,16 +14592,16 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="7"/>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="12" t="s">
         <v>594</v>
       </c>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="10"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
@@ -14761,549 +14632,549 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
+    <row r="3" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="14">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="E3" s="4">
-        <v>50</v>
-      </c>
-      <c r="F3" s="5">
-        <v>0</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="s">
+      <c r="C3" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E3" s="14">
+        <v>50</v>
+      </c>
+      <c r="F3" s="15">
+        <v>0</v>
+      </c>
+      <c r="G3" s="15">
+        <v>-1</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I3" s="14"/>
+    </row>
+    <row r="4" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="14">
+        <v>12</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E4" s="14">
+        <v>50</v>
+      </c>
+      <c r="F4" s="15">
+        <v>0</v>
+      </c>
+      <c r="G4" s="15">
+        <v>0</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="I3" s="4">
+      <c r="I4" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="14">
+        <v>15</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E5" s="14">
+        <v>50</v>
+      </c>
+      <c r="F5" s="15">
+        <v>-1</v>
+      </c>
+      <c r="G5" s="15">
+        <v>-1</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I5" s="14"/>
+    </row>
+    <row r="6" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="14">
+        <v>22</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>619</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E6" s="14">
+        <v>50</v>
+      </c>
+      <c r="F6" s="15">
+        <v>0</v>
+      </c>
+      <c r="G6" s="15">
+        <v>0</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I6" s="14"/>
+    </row>
+    <row r="7" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14">
+        <v>38</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E7" s="14">
+        <v>50</v>
+      </c>
+      <c r="F7" s="15">
+        <v>0</v>
+      </c>
+      <c r="G7" s="15">
+        <v>0</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I7" s="14"/>
+    </row>
+    <row r="8" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="14">
+        <v>46</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E8" s="14">
+        <v>50</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I8" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="14">
+        <v>50</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E9" s="14">
+        <v>50</v>
+      </c>
+      <c r="F9" s="15">
+        <v>0</v>
+      </c>
+      <c r="G9" s="15">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I9" s="14"/>
+    </row>
+    <row r="10" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="14">
+        <v>56</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>300</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E10" s="14">
+        <v>50</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I10" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="14">
+        <v>63</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E11" s="14">
+        <v>0</v>
+      </c>
+      <c r="F11" s="15">
+        <v>0</v>
+      </c>
+      <c r="G11" s="15">
+        <v>0</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I11" s="14"/>
+    </row>
+    <row r="12" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="14">
+        <v>64</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E12" s="14">
+        <v>0</v>
+      </c>
+      <c r="F12" s="15">
+        <v>0</v>
+      </c>
+      <c r="G12" s="15">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="14"/>
+    </row>
+    <row r="13" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="14">
+        <v>72</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>613</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E13" s="14">
+        <v>0</v>
+      </c>
+      <c r="F13" s="15">
+        <v>0</v>
+      </c>
+      <c r="G13" s="15">
+        <v>0</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I13" s="14"/>
+    </row>
+    <row r="14" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="14">
+        <v>73</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>597</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>634</v>
+      </c>
+      <c r="E14" s="14">
+        <v>0</v>
+      </c>
+      <c r="F14" s="15">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15">
+        <v>0</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I14" s="14"/>
+    </row>
+    <row r="15" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="14">
+        <v>4</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>604</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E15" s="14">
+        <v>50</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G15" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I15" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="14">
+        <v>17</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>612</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E16" s="14">
+        <v>50</v>
+      </c>
+      <c r="F16" s="15">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I16" s="14">
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>597</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>634</v>
-      </c>
-      <c r="E4" s="4">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0</v>
-      </c>
-      <c r="G4" s="5">
-        <v>-1</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I4" s="4"/>
-    </row>
-    <row r="5" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>598</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>637</v>
-      </c>
-      <c r="E5" s="4">
-        <v>50</v>
-      </c>
-      <c r="F5" s="5">
-        <v>-1</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I5" s="4"/>
-    </row>
-    <row r="6" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
-        <v>4</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="4" t="s">
+    <row r="17" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="14">
+        <v>19</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>612</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E17" s="14">
+        <v>50</v>
+      </c>
+      <c r="F17" s="15">
+        <v>0</v>
+      </c>
+      <c r="G17" s="15">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="I17" s="14"/>
+    </row>
+    <row r="18" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="14">
+        <v>26</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>609</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E18" s="14">
+        <v>50</v>
+      </c>
+      <c r="F18" s="15">
+        <v>0</v>
+      </c>
+      <c r="G18" s="15">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I18" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="14">
+        <v>37</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>604</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D19" s="14" t="s">
         <v>635</v>
       </c>
-      <c r="E6" s="4">
-        <v>50</v>
-      </c>
-      <c r="F6" s="4" t="s">
+      <c r="E19" s="14">
+        <v>50</v>
+      </c>
+      <c r="F19" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G19" s="15">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I19" s="14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="14">
+        <v>53</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>626</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E20" s="14">
+        <v>50</v>
+      </c>
+      <c r="F20" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="G20" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="I6" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>5</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>614</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>639</v>
-      </c>
-      <c r="E7" s="4">
-        <v>50</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="E8" s="4">
-        <v>50</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0</v>
-      </c>
-      <c r="H8" s="4" t="s">
+      <c r="I20" s="14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" s="16" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="14">
+        <v>62</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>325</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>604</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>635</v>
+      </c>
+      <c r="E21" s="14">
+        <v>50</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="I8" s="4">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>7</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>600</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>639</v>
-      </c>
-      <c r="E9" s="4">
-        <v>50</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>9</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>601</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>611</v>
-      </c>
-      <c r="E10" s="4">
-        <v>50</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <v>-1</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I10" s="4"/>
-    </row>
-    <row r="11" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>10</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>599</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>636</v>
-      </c>
-      <c r="E11" s="4">
-        <v>50</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I11" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
-        <v>11</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>639</v>
-      </c>
-      <c r="E12" s="4">
-        <v>50</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>-1</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I12" s="4"/>
-    </row>
-    <row r="13" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
-        <v>12</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>597</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>634</v>
-      </c>
-      <c r="E13" s="4">
-        <v>50</v>
-      </c>
-      <c r="F13" s="5">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I13" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4">
-        <v>13</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>596</v>
-      </c>
-      <c r="E14" s="4">
-        <v>50</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="4">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="4">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>615</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>639</v>
-      </c>
-      <c r="E15" s="4">
-        <v>50</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I15" s="4">
+      <c r="I21" s="14">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4">
-        <v>15</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>597</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>634</v>
-      </c>
-      <c r="E16" s="4">
-        <v>50</v>
-      </c>
-      <c r="F16" s="5">
-        <v>-1</v>
-      </c>
-      <c r="G16" s="5">
-        <v>-1</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="4">
-        <v>16</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>599</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>636</v>
-      </c>
-      <c r="E17" s="4">
-        <v>50</v>
-      </c>
-      <c r="F17" s="5">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I17" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A18" s="4">
-        <v>17</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>635</v>
-      </c>
-      <c r="E18" s="4">
-        <v>50</v>
-      </c>
-      <c r="F18" s="5">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5">
-        <v>0</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I18" s="4">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="4">
-        <v>19</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>635</v>
-      </c>
-      <c r="E19" s="4">
-        <v>50</v>
-      </c>
-      <c r="F19" s="5">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5">
-        <v>0</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I19" s="4"/>
-    </row>
-    <row r="20" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4">
-        <v>20</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>618</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>637</v>
-      </c>
-      <c r="E20" s="4">
-        <v>50</v>
-      </c>
-      <c r="F20" s="5">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5">
-        <v>0</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I20" s="4"/>
-    </row>
-    <row r="21" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>620</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>611</v>
-      </c>
-      <c r="E21" s="4">
-        <v>50</v>
-      </c>
-      <c r="F21" s="5">
-        <v>-1</v>
-      </c>
-      <c r="G21" s="5">
-        <v>0</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I21" s="4"/>
     </row>
     <row r="22" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>619</v>
+        <v>596</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>634</v>
+        <v>596</v>
       </c>
       <c r="E22" s="4">
         <v>50</v>
@@ -15315,22 +15186,24 @@
         <v>0</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I22" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I22" s="4">
+        <v>29</v>
+      </c>
     </row>
     <row r="23" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>11</v>
+        <v>596</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>611</v>
+        <v>596</v>
       </c>
       <c r="E23" s="4">
         <v>50</v>
@@ -15342,22 +15215,24 @@
         <v>0</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I23" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I23" s="4">
+        <v>8</v>
+      </c>
     </row>
     <row r="24" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>638</v>
+        <v>596</v>
       </c>
       <c r="E24" s="4">
         <v>50</v>
@@ -15369,9 +15244,11 @@
         <v>0</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I24" s="4"/>
+        <v>117</v>
+      </c>
+      <c r="I24" s="4">
+        <v>46</v>
+      </c>
     </row>
     <row r="25" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
@@ -15402,25 +15279,25 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>41</v>
+        <v>194</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>609</v>
+        <v>596</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>635</v>
+        <v>596</v>
       </c>
       <c r="E26" s="4">
         <v>50</v>
       </c>
-      <c r="F26" s="5">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5">
-        <v>0</v>
+      <c r="F26" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>108</v>
@@ -15431,16 +15308,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>43</v>
+        <v>198</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>602</v>
+        <v>596</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>638</v>
+        <v>596</v>
       </c>
       <c r="E27" s="4">
         <v>50</v>
@@ -15458,52 +15335,54 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>44</v>
+        <v>203</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>637</v>
+        <v>596</v>
       </c>
       <c r="E28" s="4">
         <v>50</v>
       </c>
-      <c r="F28" s="5">
-        <v>0</v>
+      <c r="F28" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G28" s="5">
         <v>0</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I28" s="4"/>
+        <v>117</v>
+      </c>
+      <c r="I28" s="4">
+        <v>43</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
-        <v>29</v>
+        <v>65</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>50</v>
+        <v>113</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>621</v>
+        <v>606</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>637</v>
+        <v>596</v>
       </c>
       <c r="E29" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F29" s="5">
         <v>0</v>
       </c>
       <c r="G29" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>109</v>
@@ -15512,19 +15391,19 @@
     </row>
     <row r="30" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>52</v>
+        <v>128</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>605</v>
+        <v>630</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>639</v>
+        <v>596</v>
       </c>
       <c r="E30" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F30" s="5">
         <v>0</v>
@@ -15539,16 +15418,16 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="4">
-        <v>31</v>
+        <v>52</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>54</v>
+        <v>235</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>605</v>
+        <v>625</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E31" s="4">
         <v>50</v>
@@ -15566,43 +15445,45 @@
     </row>
     <row r="32" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>622</v>
+        <v>599</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E32" s="4">
         <v>50</v>
       </c>
       <c r="F32" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G32" s="5">
         <v>0</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I32" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I32" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="4">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E33" s="4">
         <v>50</v>
@@ -15617,21 +15498,21 @@
         <v>108</v>
       </c>
       <c r="I33" s="4">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>59</v>
+        <v>176</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E34" s="4">
         <v>50</v>
@@ -15649,19 +15530,19 @@
     </row>
     <row r="35" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>63</v>
+        <v>137</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E35" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F35" s="5">
         <v>0</v>
@@ -15676,19 +15557,19 @@
     </row>
     <row r="36" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
-        <v>36</v>
+        <v>77</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>64</v>
+        <v>143</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>598</v>
+        <v>616</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="E36" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F36" s="5">
         <v>0</v>
@@ -15703,48 +15584,46 @@
     </row>
     <row r="37" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4">
-        <v>37</v>
+        <v>78</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>73</v>
+        <v>153</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>604</v>
+        <v>631</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="E37" s="4">
-        <v>50</v>
-      </c>
-      <c r="F37" s="4" t="s">
-        <v>110</v>
+        <v>0</v>
+      </c>
+      <c r="F37" s="5">
+        <v>0</v>
       </c>
       <c r="G37" s="5">
         <v>0</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I37" s="4">
-        <v>21</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I37" s="4"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>75</v>
+        <v>220</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="E38" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F38" s="5">
         <v>0</v>
@@ -15759,16 +15638,16 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>88</v>
+        <v>35</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E39" s="4">
         <v>50</v>
@@ -15786,16 +15665,16 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>91</v>
+        <v>43</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E40" s="4">
         <v>50</v>
@@ -15803,34 +15682,32 @@
       <c r="F40" s="5">
         <v>0</v>
       </c>
-      <c r="G40" s="4" t="s">
-        <v>110</v>
+      <c r="G40" s="5">
+        <v>0</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I40" s="4">
-        <v>0</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I40" s="4"/>
     </row>
     <row r="41" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>176</v>
+        <v>2</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E41" s="4">
         <v>50</v>
       </c>
       <c r="F41" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G41" s="5">
         <v>0</v>
@@ -15842,16 +15719,16 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>189</v>
+        <v>28</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>600</v>
+        <v>618</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E42" s="4">
         <v>50</v>
@@ -15859,25 +15736,23 @@
       <c r="F42" s="5">
         <v>0</v>
       </c>
-      <c r="G42" s="4" t="s">
-        <v>110</v>
+      <c r="G42" s="5">
+        <v>0</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I42" s="4">
-        <v>0</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I42" s="4"/>
     </row>
     <row r="43" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>191</v>
+        <v>44</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>623</v>
+        <v>598</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>637</v>
@@ -15898,16 +15773,16 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>193</v>
+        <v>50</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>600</v>
+        <v>621</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E44" s="4">
         <v>50</v>
@@ -15916,85 +15791,81 @@
         <v>0</v>
       </c>
       <c r="G44" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I44" s="4">
-        <v>29</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I44" s="4"/>
     </row>
     <row r="45" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>194</v>
+        <v>57</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>596</v>
+        <v>622</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>596</v>
+        <v>637</v>
       </c>
       <c r="E45" s="4">
         <v>50</v>
       </c>
-      <c r="F45" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>110</v>
+      <c r="F45" s="5">
+        <v>-1</v>
+      </c>
+      <c r="G45" s="5">
+        <v>0</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I45" s="4">
-        <v>0</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I45" s="4"/>
     </row>
     <row r="46" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>197</v>
+        <v>58</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>597</v>
+        <v>607</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E46" s="4">
         <v>50</v>
       </c>
-      <c r="F46" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>110</v>
+      <c r="F46" s="5">
+        <v>0</v>
+      </c>
+      <c r="G46" s="5">
+        <v>0</v>
       </c>
       <c r="H46" s="4" t="s">
         <v>108</v>
       </c>
       <c r="I46" s="4">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="4">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>198</v>
+        <v>59</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>596</v>
+        <v>637</v>
       </c>
       <c r="E47" s="4">
         <v>50</v>
@@ -16012,45 +15883,43 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="4">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>201</v>
+        <v>63</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>624</v>
+        <v>603</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E48" s="4">
         <v>50</v>
       </c>
-      <c r="F48" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>110</v>
+      <c r="F48" s="5">
+        <v>0</v>
+      </c>
+      <c r="G48" s="5">
+        <v>0</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I48" s="4">
-        <v>0</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I48" s="4"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>202</v>
+        <v>64</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>624</v>
+        <v>598</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E49" s="4">
         <v>50</v>
@@ -16059,7 +15928,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H49" s="4" t="s">
         <v>109</v>
@@ -16068,16 +15937,16 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>213</v>
+        <v>88</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E50" s="4">
         <v>50</v>
@@ -16095,16 +15964,16 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>229</v>
+        <v>91</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E51" s="4">
         <v>50</v>
@@ -16124,16 +15993,16 @@
     </row>
     <row r="52" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>235</v>
+        <v>191</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="E52" s="4">
         <v>50</v>
@@ -16151,16 +16020,16 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>255</v>
+        <v>278</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>626</v>
+        <v>603</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E53" s="4">
         <v>50</v>
@@ -16175,18 +16044,18 @@
         <v>108</v>
       </c>
       <c r="I53" s="4">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>278</v>
+        <v>72</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>603</v>
+        <v>628</v>
       </c>
       <c r="D54" s="4" t="s">
         <v>637</v>
@@ -16194,34 +16063,32 @@
       <c r="E54" s="4">
         <v>50</v>
       </c>
-      <c r="F54" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>110</v>
+      <c r="F54" s="5">
+        <v>0</v>
+      </c>
+      <c r="G54" s="5">
+        <v>0</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I54" s="4">
-        <v>29</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I54" s="4"/>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="4">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>284</v>
+        <v>119</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>627</v>
+        <v>598</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E55" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F55" s="5">
         <v>0</v>
@@ -16236,77 +16103,73 @@
     </row>
     <row r="56" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>300</v>
+        <v>127</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="E56" s="4">
-        <v>50</v>
-      </c>
-      <c r="F56" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>110</v>
+        <v>0</v>
+      </c>
+      <c r="F56" s="5">
+        <v>0</v>
+      </c>
+      <c r="G56" s="5">
+        <v>0</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I56" s="4">
-        <v>0</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I56" s="4"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="4">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>316</v>
+        <v>135</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E57" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F57" s="5">
         <v>0</v>
       </c>
-      <c r="G57" s="4" t="s">
-        <v>110</v>
+      <c r="G57" s="5">
+        <v>0</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I57" s="4">
-        <v>57</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I57" s="4"/>
     </row>
     <row r="58" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>336</v>
+        <v>159</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="E58" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F58" s="5">
         <v>0</v>
@@ -16321,19 +16184,19 @@
     </row>
     <row r="59" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="D59" s="4" t="s">
         <v>637</v>
       </c>
       <c r="E59" s="4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F59" s="5">
         <v>0</v>
@@ -16348,83 +16211,79 @@
     </row>
     <row r="60" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>203</v>
+        <v>170</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>596</v>
+        <v>637</v>
       </c>
       <c r="E60" s="4">
-        <v>50</v>
-      </c>
-      <c r="F60" s="4" t="s">
-        <v>110</v>
+        <v>0</v>
+      </c>
+      <c r="F60" s="5">
+        <v>0</v>
       </c>
       <c r="G60" s="5">
         <v>0</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="I60" s="4">
-        <v>43</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I60" s="4"/>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="4">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>325</v>
+        <v>174</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>604</v>
+        <v>633</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E61" s="4">
-        <v>50</v>
-      </c>
-      <c r="F61" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>110</v>
+        <v>0</v>
+      </c>
+      <c r="F61" s="5">
+        <v>0</v>
+      </c>
+      <c r="G61" s="5">
+        <v>0</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="I61" s="4">
-        <v>29</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="I61" s="4"/>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" s="4">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>111</v>
+        <v>11</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>613</v>
+        <v>601</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>634</v>
+        <v>611</v>
       </c>
       <c r="E62" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F62" s="5">
         <v>0</v>
       </c>
       <c r="G62" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H62" s="4" t="s">
         <v>109</v>
@@ -16433,22 +16292,22 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>634</v>
+        <v>611</v>
       </c>
       <c r="E63" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F63" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G63" s="5">
         <v>0</v>
@@ -16460,19 +16319,19 @@
     </row>
     <row r="64" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>113</v>
+        <v>34</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>606</v>
+        <v>11</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="E64" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F64" s="5">
         <v>0</v>
@@ -16487,10 +16346,10 @@
     </row>
     <row r="65" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>114</v>
+        <v>7</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>614</v>
@@ -16499,7 +16358,7 @@
         <v>639</v>
       </c>
       <c r="E65" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F65" s="5">
         <v>0</v>
@@ -16514,19 +16373,19 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" s="4">
-        <v>67</v>
+        <v>7</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>119</v>
+        <v>9</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E66" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F66" s="5">
         <v>0</v>
@@ -16541,25 +16400,25 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" s="4">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>123</v>
+        <v>13</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>624</v>
+        <v>615</v>
       </c>
       <c r="D67" s="4" t="s">
         <v>639</v>
       </c>
       <c r="E67" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F67" s="5">
         <v>0</v>
       </c>
       <c r="G67" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H67" s="4" t="s">
         <v>109</v>
@@ -16568,46 +16427,48 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" s="4">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>126</v>
+        <v>18</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>629</v>
+        <v>615</v>
       </c>
       <c r="D68" s="4" t="s">
         <v>639</v>
       </c>
       <c r="E68" s="4">
-        <v>0</v>
-      </c>
-      <c r="F68" s="5">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="G68" s="5">
         <v>0</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I68" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I68" s="4">
+        <v>29</v>
+      </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" s="4">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>127</v>
+        <v>52</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E69" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F69" s="5">
         <v>0</v>
@@ -16622,19 +16483,19 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>128</v>
+        <v>54</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>630</v>
+        <v>605</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>596</v>
+        <v>639</v>
       </c>
       <c r="E70" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F70" s="5">
         <v>0</v>
@@ -16649,46 +16510,48 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>129</v>
+        <v>189</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>613</v>
+        <v>600</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="E71" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F71" s="5">
         <v>0</v>
       </c>
-      <c r="G71" s="5">
-        <v>0</v>
+      <c r="G71" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I71" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I71" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" s="4">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>132</v>
+        <v>193</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="E72" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F72" s="5">
         <v>0</v>
@@ -16697,58 +16560,62 @@
         <v>0</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I72" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I72" s="4">
+        <v>29</v>
+      </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>135</v>
+        <v>201</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>598</v>
+        <v>624</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E73" s="4">
-        <v>0</v>
-      </c>
-      <c r="F73" s="5">
-        <v>0</v>
-      </c>
-      <c r="G73" s="5">
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I73" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I73" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="74" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>137</v>
+        <v>202</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>599</v>
+        <v>624</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E74" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F74" s="5">
         <v>0</v>
       </c>
       <c r="G74" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H74" s="4" t="s">
         <v>109</v>
@@ -16757,46 +16624,48 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" s="4">
-        <v>76</v>
+        <v>51</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>139</v>
+        <v>229</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>615</v>
+        <v>600</v>
       </c>
       <c r="D75" s="4" t="s">
         <v>639</v>
       </c>
       <c r="E75" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F75" s="5">
         <v>0</v>
       </c>
-      <c r="G75" s="5">
-        <v>0</v>
+      <c r="G75" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I75" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="I75" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="76" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>143</v>
+        <v>284</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E76" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F76" s="5">
         <v>0</v>
@@ -16811,46 +16680,48 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>153</v>
+        <v>316</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>631</v>
+        <v>600</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E77" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F77" s="5">
         <v>0</v>
       </c>
-      <c r="G77" s="5">
-        <v>0</v>
+      <c r="G77" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="I77" s="4"/>
+        <v>117</v>
+      </c>
+      <c r="I77" s="4">
+        <v>57</v>
+      </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" s="4">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>159</v>
+        <v>336</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>608</v>
+        <v>600</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E78" s="4">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F78" s="5">
         <v>0</v>
@@ -16865,16 +16736,16 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>166</v>
+        <v>114</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>632</v>
+        <v>614</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E79" s="4">
         <v>0</v>
@@ -16892,16 +16763,16 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" s="4">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>170</v>
+        <v>123</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>598</v>
+        <v>624</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E80" s="4">
         <v>0</v>
@@ -16919,16 +16790,16 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>174</v>
+        <v>126</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E81" s="4">
         <v>0</v>
@@ -16946,16 +16817,16 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82" s="4">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>220</v>
+        <v>139</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>599</v>
+        <v>615</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E82" s="4">
         <v>0</v>
@@ -16974,7 +16845,7 @@
   </sheetData>
   <autoFilter ref="A2:I82" xr:uid="{B4B83C6E-BA35-4A1C-B7DF-FEE986A0867B}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:I82">
-      <sortCondition ref="A2:A82"/>
+      <sortCondition ref="D2:D82"/>
     </sortState>
   </autoFilter>
   <mergeCells count="1">
@@ -16985,16 +16856,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F401B0B-95D1-474E-9F7E-7852CE4031B8}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30180552-B278-41A7-8750-56B4914963F1}">
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -17020,10 +16881,10 @@
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="13" t="s">
         <v>645</v>
       </c>
-      <c r="B6" s="12"/>
+      <c r="B6" s="13"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
@@ -17074,10 +16935,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="10" t="s">
         <v>636</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="10">
         <v>7</v>
       </c>
     </row>

</xml_diff>